<commit_message>
matrix: fix Ozon channel eligibility (Celimax/Round Lab/Ded Moroz/robots only)
Ozon sells only Ded Moroz, robots (compute), and Celimax + Round Lab cosmetics;
all other cosmetics (incl. FARMSTAY) are WB-only (no docs / no demand / price).
Added "Где продавать" column reflecting this.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/matrix/polnaya_kartina_plus_spros_2026.xlsx
+++ b/outputs/matrix/polnaya_kartina_plus_spros_2026.xlsx
@@ -459,22 +459,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M143"/>
+  <dimension ref="A1:N143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,7 +501,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ВСЕГО шт (склад+конт+маш)</t>
+          <t>ВСЕГО шт</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -539,6 +540,11 @@
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Где продавать</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ВЕРДИКТ</t>
         </is>
@@ -589,9 +595,14 @@
       <c r="L2" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (19 мес) → не докупать, распродавать</t>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>ЗАТОВАРЕН (19 мес) → не докупать</t>
         </is>
       </c>
     </row>
@@ -642,6 +653,11 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -693,6 +709,11 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -731,10 +752,10 @@
         <v>1124.6</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1126.9</v>
+        <v>1124.6</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>6.5</v>
@@ -744,6 +765,11 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -782,19 +808,24 @@
         <v>1843.4</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1846.4</v>
+        <v>1843.4</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>146</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -846,6 +877,11 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -897,6 +933,11 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -947,6 +988,11 @@
         <v>38</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -995,7 +1041,12 @@
       <c r="L10" s="2" t="n">
         <v>-31</v>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -1046,7 +1097,12 @@
       <c r="L11" s="2" t="n">
         <v>112</v>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -1086,19 +1142,24 @@
         <v>107.1</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>112.8</v>
+        <v>107.1</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>99</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -1137,10 +1198,10 @@
         <v>1745.7</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>1746.4</v>
+        <v>1745.7</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>4.2</v>
@@ -1150,6 +1211,11 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -1201,6 +1267,11 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -1250,7 +1321,12 @@
       <c r="L15" s="2" t="n">
         <v>-266</v>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -1303,6 +1379,11 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -1352,9 +1433,14 @@
       <c r="L17" s="2" t="n">
         <v>135</v>
       </c>
-      <c r="M17" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (129 мес) → не докупать, распродавать</t>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>ЗАТОВАРЕН (129 мес) → не докупать</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1481,12 @@
       </c>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1447,6 +1538,11 @@
         <v>43</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -1489,7 +1585,12 @@
       </c>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1529,10 +1630,10 @@
         <v>282.1</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>283.1</v>
+        <v>282.1</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>3.3</v>
@@ -1541,6 +1642,11 @@
         <v>30</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -1583,7 +1689,12 @@
       </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1626,7 +1737,12 @@
       </c>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1677,7 +1793,12 @@
       <c r="L24" s="2" t="n">
         <v>-72</v>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -1720,7 +1841,12 @@
       </c>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1763,7 +1889,12 @@
       </c>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1806,7 +1937,12 @@
       </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1849,7 +1985,12 @@
       </c>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -1889,18 +2030,23 @@
         <v>22.7</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>7.3</v>
+        <v>0</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>30</v>
+        <v>22.7</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>20.4</v>
+        <v>27</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>-370</v>
       </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -1936,18 +2082,21 @@
         <v>0</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K30" s="2" t="n">
-        <v>200</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (200 мес) → не докупать, распродавать</t>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>нет продаж → распродать</t>
         </is>
       </c>
     </row>
@@ -1998,6 +2147,11 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -2036,19 +2190,24 @@
         <v>36.7</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>42.4</v>
+        <v>36.7</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>15.3</v>
+        <v>17.7</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>57</v>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -2087,18 +2246,23 @@
         <v>82.09999999999999</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>88.09999999999999</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -2141,7 +2305,12 @@
       </c>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2192,9 +2361,14 @@
       <c r="L35" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (18 мес) → не докупать, распродавать</t>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>ЗАТОВАРЕН (18 мес) → не докупать</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2409,12 @@
       </c>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2278,7 +2457,12 @@
       </c>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2321,7 +2505,12 @@
       </c>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2373,6 +2562,11 @@
         <v>16</v>
       </c>
       <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -2415,7 +2609,12 @@
       </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="4" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2455,10 +2654,10 @@
         <v>347.4</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>350.1</v>
+        <v>347.4</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>2.6</v>
@@ -2466,7 +2665,12 @@
       <c r="L41" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="M41" s="5" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -2506,18 +2710,21 @@
         <v>0</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K42" s="2" t="n">
-        <v>198.5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="n">
         <v>-308</v>
       </c>
-      <c r="M42" s="4" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -2570,6 +2777,11 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -2608,18 +2820,23 @@
         <v>149.3</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>149.6</v>
+        <v>149.3</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>9.4</v>
+        <v>9.5</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>-8</v>
       </c>
-      <c r="M44" s="4" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -2671,6 +2888,11 @@
         <v>6</v>
       </c>
       <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -2713,7 +2935,12 @@
       </c>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
-      <c r="M46" s="4" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2753,19 +2980,24 @@
         <v>170.9</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>172.9</v>
+        <v>170.9</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>34</v>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -2815,7 +3047,12 @@
       <c r="L48" s="2" t="n">
         <v>-8</v>
       </c>
-      <c r="M48" s="4" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N48" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -2858,7 +3095,12 @@
       </c>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr">
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -2910,6 +3152,11 @@
         <v>19</v>
       </c>
       <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -2952,7 +3199,12 @@
       </c>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3004,6 +3256,11 @@
         <v>32</v>
       </c>
       <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -3046,7 +3303,12 @@
       </c>
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr"/>
-      <c r="M53" s="4" t="inlineStr">
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3089,7 +3351,12 @@
       </c>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
-      <c r="M54" s="4" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3141,6 +3408,11 @@
         <v>10</v>
       </c>
       <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -3183,7 +3455,12 @@
       </c>
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr"/>
-      <c r="M56" s="4" t="inlineStr">
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3236,6 +3513,11 @@
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -3274,10 +3556,10 @@
         <v>371.7</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>373.7</v>
+        <v>371.7</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>2.3</v>
@@ -3285,7 +3567,12 @@
       <c r="L58" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="M58" s="5" t="inlineStr">
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N58" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -3337,6 +3624,11 @@
         <v>19</v>
       </c>
       <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -3379,7 +3671,12 @@
       </c>
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
-      <c r="M60" s="4" t="inlineStr">
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3430,9 +3727,14 @@
       <c r="L61" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="M61" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (120 мес) → не докупать, распродавать</t>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="inlineStr">
+        <is>
+          <t>ЗАТОВАРЕН (120 мес) → не докупать</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3775,12 @@
       </c>
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
-      <c r="M62" s="4" t="inlineStr">
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3516,7 +3823,12 @@
       </c>
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr"/>
-      <c r="M63" s="4" t="inlineStr">
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3569,6 +3881,11 @@
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -3619,6 +3936,11 @@
         <v>55</v>
       </c>
       <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -3661,7 +3983,12 @@
       </c>
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr"/>
-      <c r="M66" s="4" t="inlineStr">
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3704,7 +4031,12 @@
       </c>
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr"/>
-      <c r="M67" s="4" t="inlineStr">
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3747,7 +4079,12 @@
       </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
-      <c r="M68" s="4" t="inlineStr">
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3790,7 +4127,12 @@
       </c>
       <c r="K69" s="2" t="inlineStr"/>
       <c r="L69" s="2" t="inlineStr"/>
-      <c r="M69" s="4" t="inlineStr">
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3841,7 +4183,12 @@
       <c r="L70" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="M70" s="5" t="inlineStr">
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -3884,7 +4231,12 @@
       </c>
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr"/>
-      <c r="M71" s="4" t="inlineStr">
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N71" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -3935,7 +4287,12 @@
       <c r="L72" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="M72" s="5" t="inlineStr">
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N72" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -3978,7 +4335,12 @@
       </c>
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr"/>
-      <c r="M73" s="4" t="inlineStr">
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4021,7 +4383,12 @@
       </c>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr"/>
-      <c r="M74" s="4" t="inlineStr">
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N74" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4064,7 +4431,12 @@
       </c>
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr"/>
-      <c r="M75" s="4" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4117,6 +4489,11 @@
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -4155,10 +4532,10 @@
         <v>69.7</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>70.40000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>5.8</v>
@@ -4167,6 +4544,11 @@
         <v>40</v>
       </c>
       <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -4211,6 +4593,11 @@
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -4260,7 +4647,12 @@
       <c r="L79" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="M79" s="5" t="inlineStr">
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N79" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -4305,7 +4697,12 @@
         <v>0.7</v>
       </c>
       <c r="L80" s="2" t="inlineStr"/>
-      <c r="M80" s="5" t="inlineStr">
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N80" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -4348,7 +4745,12 @@
       </c>
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr"/>
-      <c r="M81" s="4" t="inlineStr">
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4400,6 +4802,11 @@
         <v>12</v>
       </c>
       <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -4442,7 +4849,12 @@
       </c>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
-      <c r="M83" s="4" t="inlineStr">
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4485,7 +4897,12 @@
       </c>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
-      <c r="M84" s="4" t="inlineStr">
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4537,6 +4954,11 @@
         <v>49</v>
       </c>
       <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -4579,7 +5001,12 @@
       </c>
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
-      <c r="M86" s="4" t="inlineStr">
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N86" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4622,7 +5049,12 @@
       </c>
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr"/>
-      <c r="M87" s="4" t="inlineStr">
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N87" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4674,6 +5106,11 @@
         <v>67</v>
       </c>
       <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
         <is>
           <t>норма</t>
         </is>
@@ -4718,6 +5155,11 @@
       <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -4759,7 +5201,12 @@
       </c>
       <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr"/>
-      <c r="M90" s="4" t="inlineStr">
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N90" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4812,6 +5259,11 @@
       </c>
       <c r="M91" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -4861,7 +5313,12 @@
       <c r="L92" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="M92" s="5" t="inlineStr">
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N92" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -4904,7 +5361,12 @@
       </c>
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr"/>
-      <c r="M93" s="4" t="inlineStr">
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N93" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -4955,7 +5417,12 @@
       <c r="L94" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="M94" s="5" t="inlineStr">
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N94" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -4995,20 +5462,25 @@
         <v>33.4</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>34.1</v>
+        <v>33.4</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>20.8</v>
+        <v>21.2</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="M95" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (21 мес) → не докупать, распродавать</t>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N95" s="3" t="inlineStr">
+        <is>
+          <t>ЗАТОВАРЕН (21 мес) → не докупать</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5529,12 @@
       <c r="L96" s="2" t="n">
         <v>-97</v>
       </c>
-      <c r="M96" s="4" t="inlineStr">
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N96" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -5100,7 +5577,12 @@
       </c>
       <c r="K97" s="2" t="inlineStr"/>
       <c r="L97" s="2" t="inlineStr"/>
-      <c r="M97" s="4" t="inlineStr">
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N97" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -5140,10 +5622,10 @@
         <v>174.9</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>175.6</v>
+        <v>174.9</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>1.4</v>
@@ -5151,7 +5633,12 @@
       <c r="L98" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="M98" s="5" t="inlineStr">
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N98" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -5194,7 +5681,12 @@
       </c>
       <c r="K99" s="2" t="inlineStr"/>
       <c r="L99" s="2" t="inlineStr"/>
-      <c r="M99" s="4" t="inlineStr">
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N99" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>
@@ -5234,19 +5726,24 @@
         <v>45</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>45.7</v>
+        <v>45</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>14.3</v>
+        <v>14.5</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>143</v>
       </c>
       <c r="M100" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5296,7 +5793,12 @@
       <c r="L101" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="M101" s="4" t="inlineStr">
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N101" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -5349,6 +5851,11 @@
       </c>
       <c r="M102" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5398,9 +5905,14 @@
       <c r="L103" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="M103" s="3" t="inlineStr">
-        <is>
-          <t>ЗАТОВАРЕН (31 мес) → не докупать, распродавать</t>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr">
+        <is>
+          <t>ЗАТОВАРЕН (31 мес) → не докупать</t>
         </is>
       </c>
     </row>
@@ -5438,19 +5950,24 @@
         <v>19.9</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>20.6</v>
+        <v>19.9</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>38</v>
       </c>
       <c r="M104" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5489,19 +6006,24 @@
         <v>116.6</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>116.9</v>
+        <v>116.6</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>34</v>
       </c>
       <c r="M105" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5540,19 +6062,24 @@
         <v>66.09999999999999</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>66.8</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>151</v>
       </c>
       <c r="M106" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5604,6 +6131,11 @@
       </c>
       <c r="M107" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5642,19 +6174,24 @@
         <v>20</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>20.7</v>
+        <v>20</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>16</v>
       </c>
       <c r="M108" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5693,10 +6230,10 @@
         <v>69.40000000000001</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>69.7</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>5.8</v>
@@ -5706,6 +6243,11 @@
       </c>
       <c r="M109" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5755,7 +6297,12 @@
       <c r="L110" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="M110" s="5" t="inlineStr">
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N110" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -5806,7 +6353,12 @@
       <c r="L111" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="M111" s="5" t="inlineStr">
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N111" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -5851,6 +6403,11 @@
       <c r="L112" s="2" t="inlineStr"/>
       <c r="M112" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5902,6 +6459,11 @@
       </c>
       <c r="M113" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -5940,18 +6502,23 @@
         <v>6.9</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>25.7</v>
+        <v>0</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>32.6</v>
+        <v>6.9</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>1.7</v>
+        <v>8</v>
       </c>
       <c r="L114" s="2" t="inlineStr"/>
-      <c r="M114" s="5" t="inlineStr">
-        <is>
-          <t>ДЕФИЦИТ → докупать/следить</t>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>норма</t>
         </is>
       </c>
     </row>
@@ -6002,6 +6569,11 @@
       </c>
       <c r="M115" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6053,6 +6625,11 @@
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6104,6 +6681,11 @@
       </c>
       <c r="M117" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6142,10 +6724,10 @@
         <v>149.1</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>150.1</v>
+        <v>149.1</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>1.2</v>
@@ -6153,7 +6735,12 @@
       <c r="L118" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="M118" s="5" t="inlineStr">
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N118" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6193,10 +6780,10 @@
         <v>129.7</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>130.4</v>
+        <v>129.7</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>1.6</v>
@@ -6204,7 +6791,12 @@
       <c r="L119" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="M119" s="5" t="inlineStr">
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N119" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6244,10 +6836,10 @@
         <v>276.6</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>277.3</v>
+        <v>276.6</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0.8</v>
@@ -6255,7 +6847,12 @@
       <c r="L120" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="M120" s="5" t="inlineStr">
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N120" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6308,6 +6905,11 @@
       </c>
       <c r="M121" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N121" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6346,19 +6948,24 @@
         <v>22.9</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>23.9</v>
+        <v>22.9</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>17.2</v>
+        <v>17.9</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>144</v>
       </c>
       <c r="M122" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6408,7 +7015,12 @@
       <c r="L123" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M123" s="4" t="inlineStr">
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N123" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -6459,7 +7071,12 @@
       <c r="L124" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="M124" s="5" t="inlineStr">
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N124" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6510,7 +7127,12 @@
       <c r="L125" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="M125" s="5" t="inlineStr">
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N125" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6561,7 +7183,12 @@
       <c r="L126" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="M126" s="5" t="inlineStr">
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N126" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6612,7 +7239,12 @@
       <c r="L127" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M127" s="5" t="inlineStr">
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N127" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6665,6 +7297,11 @@
       </c>
       <c r="M128" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6703,18 +7340,23 @@
         <v>3.9</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>11.8</v>
+        <v>12.8</v>
       </c>
       <c r="L129" s="2" t="n">
         <v>-37</v>
       </c>
-      <c r="M129" s="4" t="inlineStr">
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N129" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -6767,6 +7409,11 @@
       </c>
       <c r="M130" s="2" t="inlineStr">
         <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N130" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -6816,7 +7463,12 @@
       <c r="L131" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="M131" s="5" t="inlineStr">
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N131" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6867,7 +7519,12 @@
       <c r="L132" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="M132" s="5" t="inlineStr">
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N132" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6918,7 +7575,12 @@
       <c r="L133" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="M133" s="5" t="inlineStr">
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N133" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -6969,7 +7631,12 @@
       <c r="L134" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="M134" s="5" t="inlineStr">
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N134" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -7020,7 +7687,12 @@
       <c r="L135" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="M135" s="5" t="inlineStr">
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>WB + Ozon</t>
+        </is>
+      </c>
+      <c r="N135" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -7060,10 +7732,10 @@
         <v>73.90000000000001</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>76.2</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>0.2</v>
@@ -7071,7 +7743,12 @@
       <c r="L136" s="2" t="n">
         <v>108</v>
       </c>
-      <c r="M136" s="5" t="inlineStr">
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N136" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -7124,6 +7801,11 @@
       </c>
       <c r="M137" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N137" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -7173,7 +7855,12 @@
       <c r="L138" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="M138" s="5" t="inlineStr">
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N138" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -7224,7 +7911,12 @@
       <c r="L139" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="M139" s="5" t="inlineStr">
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N139" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -7264,18 +7956,23 @@
         <v>16.4</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>17.1</v>
+        <v>16.4</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="L140" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="M140" s="5" t="inlineStr">
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N140" s="5" t="inlineStr">
         <is>
           <t>ДЕФИЦИТ → докупать/следить</t>
         </is>
@@ -7324,6 +8021,11 @@
       </c>
       <c r="M141" s="2" t="inlineStr">
         <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N141" s="2" t="inlineStr">
+        <is>
           <t>норма</t>
         </is>
       </c>
@@ -7373,7 +8075,12 @@
       <c r="L142" s="2" t="n">
         <v>-8</v>
       </c>
-      <c r="M142" s="4" t="inlineStr">
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N142" s="4" t="inlineStr">
         <is>
           <t>УБЫТОК → распродать/поднять цену</t>
         </is>
@@ -7412,7 +8119,12 @@
       </c>
       <c r="K143" s="2" t="inlineStr"/>
       <c r="L143" s="2" t="inlineStr"/>
-      <c r="M143" s="4" t="inlineStr">
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>только WB</t>
+        </is>
+      </c>
+      <c r="N143" s="4" t="inlineStr">
         <is>
           <t>нет продаж → распродать</t>
         </is>

</xml_diff>